<commit_message>
release smart trust v1.5.0
</commit_message>
<xml_diff>
--- a/trust/CodeSystem-Actors.xlsx
+++ b/trust/CodeSystem-Actors.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.4.0</t>
+    <t>1.5.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-11T14:17:30+00:00</t>
+    <t>2026-04-27T07:32:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>